<commit_message>
feat: identify salary by notation to group multi-currency payments
</commit_message>
<xml_diff>
--- a/test/phpunit/fixtures/valid_import.xlsx
+++ b/test/phpunit/fixtures/valid_import.xlsx
@@ -15,7 +15,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
+  <si>
+    <t>Salaire</t>
+  </si>
+  <si>
+    <t>Réf paiement</t>
+  </si>
   <si>
     <t>Prénom</t>
   </si>
@@ -26,12 +32,21 @@
     <t>Date de paiement</t>
   </si>
   <si>
-    <t>Montant</t>
-  </si>
-  <si>
     <t>Type de paiement</t>
   </si>
   <si>
+    <t>Compte bancaire</t>
+  </si>
+  <si>
+    <t>Montant payé</t>
+  </si>
+  <si>
+    <t>Montant CHF</t>
+  </si>
+  <si>
+    <t>Salaire total CHF</t>
+  </si>
+  <si>
     <t>Libellé</t>
   </si>
   <si>
@@ -44,7 +59,10 @@
     <t>Payé</t>
   </si>
   <si>
-    <t>Compte bancaire</t>
+    <t>2026-01-1</t>
+  </si>
+  <si>
+    <t>2026-01-1-CHF</t>
   </si>
   <si>
     <t>Jean</t>
@@ -56,13 +74,19 @@
     <t>VIR</t>
   </si>
   <si>
+    <t>POSTE_CH</t>
+  </si>
+  <si>
     <t>Salaire Janvier 2026</t>
   </si>
   <si>
     <t>oui</t>
   </si>
   <si>
-    <t>POSTE_CH</t>
+    <t>2026-01-2</t>
+  </si>
+  <si>
+    <t>2026-01-2-CHF</t>
   </si>
   <si>
     <t>Marie</t>
@@ -71,10 +95,22 @@
     <t>Martin</t>
   </si>
   <si>
+    <t>2026-01-3</t>
+  </si>
+  <si>
+    <t>2026-01-3-CHF</t>
+  </si>
+  <si>
     <t>Pierre</t>
   </si>
   <si>
     <t>Durand</t>
+  </si>
+  <si>
+    <t>2026-02-4</t>
+  </si>
+  <si>
+    <t>2026-02-4-CHF</t>
   </si>
   <si>
     <t>Sophie</t>
@@ -430,22 +466,26 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.140869" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="10.568848" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="19.995117" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="9.283447" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="11.711426" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="16.424561" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="8.140869" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="10.568848" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="19.995117" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="24.708252" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="13.996582" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="5.855713" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="18.709717" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="19.995117" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="18.709717" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15.281982" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="13.996582" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="21.137695" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="24.708252" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="16.424561" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="13.996582" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="5.855713" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:14">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
@@ -476,133 +516,193 @@
       <c r="J1" s="0" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:14">
       <c r="A2" s="0" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="1">
+        <v>15</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1">
         <v>46053</v>
       </c>
-      <c r="D2" s="0">
+      <c r="F2" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="0">
         <v>2500.0</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="1">
+      <c r="I2" s="0">
+        <v>2500.0</v>
+      </c>
+      <c r="J2" s="0">
+        <v>2500.0</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1">
         <v>46023</v>
       </c>
-      <c r="H2" s="1">
+      <c r="M2" s="1">
         <v>46053</v>
       </c>
-      <c r="I2" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>15</v>
+      <c r="N2" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:14">
       <c r="A3" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="1">
+        <v>23</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="1">
         <v>46053</v>
       </c>
-      <c r="D3" s="0">
+      <c r="F3" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="0">
         <v>2800.5</v>
       </c>
-      <c r="E3" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1">
+      <c r="I3" s="0">
+        <v>2800.5</v>
+      </c>
+      <c r="J3" s="0">
+        <v>2800.5</v>
+      </c>
+      <c r="K3" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="1">
         <v>46023</v>
       </c>
-      <c r="H3" s="1">
+      <c r="M3" s="1">
         <v>46053</v>
       </c>
-      <c r="I3" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="0" t="s">
-        <v>15</v>
+      <c r="N3" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:14">
       <c r="A4" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="1">
+        <v>46053</v>
+      </c>
+      <c r="F4" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="G4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="1">
+      <c r="H4" s="0">
+        <v>2200.0</v>
+      </c>
+      <c r="I4" s="0">
+        <v>2200.0</v>
+      </c>
+      <c r="J4" s="0">
+        <v>2200.0</v>
+      </c>
+      <c r="K4" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="1">
+        <v>46023</v>
+      </c>
+      <c r="M4" s="1">
         <v>46053</v>
       </c>
-      <c r="D4" s="0">
-        <v>2200.0</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="1">
-        <v>46023</v>
-      </c>
-      <c r="H4" s="1">
-        <v>46053</v>
-      </c>
-      <c r="I4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="0" t="s">
-        <v>15</v>
+      <c r="N4" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:14">
       <c r="A5" s="0" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1">
+        <v>31</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="1">
         <v>46081</v>
       </c>
-      <c r="D5" s="0">
+      <c r="F5" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="0">
         <v>3100.75</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="1">
+      <c r="I5" s="0">
+        <v>3100.75</v>
+      </c>
+      <c r="J5" s="0">
+        <v>3100.75</v>
+      </c>
+      <c r="K5" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="1">
         <v>46054</v>
       </c>
-      <c r="H5" s="1">
+      <c r="M5" s="1">
         <v>46081</v>
       </c>
-      <c r="I5" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" s="0" t="s">
-        <v>15</v>
+      <c r="N5" s="0" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>